<commit_message>
Chinh sua file thong qua url
</commit_message>
<xml_diff>
--- a/templates/BaoCao.xlsx
+++ b/templates/BaoCao.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="61">
   <si>
     <t>const docxConverter = require("docx-pdf");</t>
   </si>
@@ -44,16 +44,172 @@
     <t>pdfkit</t>
   </si>
   <si>
+    <t>Cấu trúc xml riêng để tạo pdf</t>
+  </si>
+  <si>
     <t>aspose/words</t>
   </si>
   <si>
     <t>File bị dính logo</t>
   </si>
   <si>
+    <t>&lt;pdf&gt;</t>
+  </si>
+  <si>
     <t>nutrient-sdk/node</t>
   </si>
   <si>
-    <t>Không thể dùng được bị lỗi length</t>
+    <t>Không thể dùng được bị lỗi length, phải có giấy phép</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  &lt;config&gt;</t>
+  </si>
+  <si>
+    <t>docx2pdf-converter</t>
+  </si>
+  <si>
+    <t>Phải có libre office</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;filename&gt;my-file.pdf&lt;/filename&gt;</t>
+  </si>
+  <si>
+    <t>docx-to-pdf-axios</t>
+  </si>
+  <si>
+    <t>Phải có giấy phép</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;document size="A4" marginBottom="50"/&gt;</t>
+  </si>
+  <si>
+    <t>next-doc2pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;title&gt;{{title}}&lt;/title&gt;</t>
+  </si>
+  <si>
+    <t>docx2pdf-cli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;colors darkred="#800"/&gt;</t>
+  </si>
+  <si>
+    <t>PDF Services Node.js SDK</t>
+  </si>
+  <si>
+    <t>Có phí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;styles&gt;</t>
+  </si>
+  <si>
+    <t>office-text-extractor</t>
+  </si>
+  <si>
+    <t>chuyển đổi text</t>
+  </si>
+  <si>
+    <t>pdflib</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;/styles&gt;</t>
+  </si>
+  <si>
+    <t>officeparser</t>
+  </si>
+  <si>
+    <t>Đọc text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  &lt;/config&gt;</t>
+  </si>
+  <si>
+    <t>xml-to-pdf</t>
+  </si>
+  <si>
+    <t>Theo cấu trúc xml riêng, không dựa trên xml word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  &lt;page&gt;</t>
+  </si>
+  <si>
+    <t>xml2pdf</t>
+  </si>
+  <si>
+    <t>Không dùng theo cấu trúc word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;h1&gt;{{title}}&lt;/h1&gt;</t>
+  </si>
+  <si>
+    <t>draw.io-export</t>
+  </si>
+  <si>
+    <t>Sơ đồ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;h2&gt;Page 1&lt;/h2&gt;</t>
+  </si>
+  <si>
+    <t>xml-pdf</t>
+  </si>
+  <si>
+    <t>Xml tự định nghĩa theo cấu trúc web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;indent&gt;</t>
+  </si>
+  <si>
+    <t>fast-xml-parser</t>
+  </si>
+  <si>
+    <t>Đọc xml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      &lt;p&gt;Indented text&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>docx2pdf</t>
+  </si>
+  <si>
+    <t>Phải có microft word hoặc libre office</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;/indent&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;hr thickness="6"/&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;row&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      &lt;column width="33%"&gt;Column 1&lt;/column&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      &lt;column width="66%"&gt;Column 2&lt;/column&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;/row&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;div&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        A link to &lt;a&gt;example.com&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;/div&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  &lt;/page&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;h1 top="33%" left="100"&gt;Page 2&lt;/h1&gt;</t>
+  </si>
+  <si>
+    <t>&lt;/pdf&gt;</t>
   </si>
 </sst>
 </file>
@@ -66,7 +222,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -75,8 +231,39 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="10.5"/>
-      <color rgb="FFCE9178"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Consolas"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
@@ -419,12 +606,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -545,141 +747,171 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -961,16 +1193,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>551815</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>247015</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>55880</xdr:rowOff>
+      <xdr:rowOff>93980</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -987,7 +1219,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5097780" y="182880"/>
+          <a:off x="5920740" y="220980"/>
           <a:ext cx="2380615" cy="1884680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1254,53 +1486,289 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A2:B16"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <dimension ref="A2:I43"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="38.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="43.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:9">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
+    <row r="13" spans="1:9">
+      <c r="A13" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
+    <row r="14" spans="1:9">
+      <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="1" t="s">
+      <c r="I14" t="s">
         <v>5</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="15" ht="15.6" spans="1:9">
+      <c r="A15" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="1" t="s">
+      <c r="B15" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B16" t="s">
+      <c r="I15" s="5" t="s">
         <v>8</v>
       </c>
     </row>
+    <row r="16" ht="15.6" spans="1:9">
+      <c r="A16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" ht="15.6" spans="1:9">
+      <c r="A17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" ht="15.6" spans="1:9">
+      <c r="A18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" ht="15.6" spans="1:9">
+      <c r="A19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" ht="15.6" spans="1:9">
+      <c r="A20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" ht="15.6" spans="1:9">
+      <c r="A21" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" ht="15.6" spans="1:9">
+      <c r="A23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" ht="15.6" spans="1:9">
+      <c r="A24" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" ht="15.6" spans="1:9">
+      <c r="A25" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" ht="15.6" spans="1:9">
+      <c r="A26" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" ht="15.6" spans="1:9">
+      <c r="A27" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" ht="15.6" spans="1:9">
+      <c r="A28" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" ht="15.6" spans="1:9">
+      <c r="A29" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" ht="15.6" spans="1:9">
+      <c r="A30" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" ht="15.6" spans="1:9">
+      <c r="A31" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="32" ht="15.6" spans="1:9">
+      <c r="I32" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" ht="15.6" spans="9:9">
+      <c r="I33" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" ht="15.6" spans="9:9">
+      <c r="I34" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="35" ht="15.6" spans="9:9">
+      <c r="I35" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="36" ht="15.6" spans="9:9">
+      <c r="I36" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="37" ht="15.6" spans="9:9">
+      <c r="I37" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="38" ht="15.6" spans="9:9">
+      <c r="I38" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" ht="15.6" spans="9:9">
+      <c r="I39" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40" ht="15.6" spans="9:9">
+      <c r="I40" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" ht="15.6" spans="9:9">
+      <c r="I41" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" ht="15.6" spans="9:9">
+      <c r="I42" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43" ht="15.6" spans="9:9">
+      <c r="I43" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A20" r:id="rId2" display="docx2pdf-cli" tooltip="https://www.npmjs.com/package/docx2pdf-cli"/>
+    <hyperlink ref="A29" r:id="rId3" display="fast-xml-parser" tooltip="https://www.npmjs.com/package/fast-xml-parser"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>

</xml_diff>